<commit_message>
DeviceUse: excel file refreshed
</commit_message>
<xml_diff>
--- a/input/requirements/DeviceUse.xlsx
+++ b/input/requirements/DeviceUse.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\GBB-IG\input\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MichalCiszewski\Documents\Github\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAF2FBE8-D620-4C61-A2B0-53FF1456C858}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62246BE6-3BA6-4081-A4F7-0E4AB2677F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -50,11 +50,11 @@
   <commentList>
     <comment ref="C10" authorId="0" shapeId="0" xr:uid="{34562484-290B-4F2D-9790-FE82BD1E616C}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Of, is dit concept wel bedoelt voor aanlevering LIR? Het zou wel kunnen, maar dan hebben we het over een andere use case dan zorg-zorg. We hebben het dan over zorg-overheid. bestaat zon use case al?
-Beantwoorden:
+Reply:
     Zowel de bouwblokken Device als DeviceUse zijn nodig voor LIR</t>
       </text>
     </comment>
@@ -73,33 +73,33 @@
   <commentList>
     <comment ref="I11" authorId="0" shapeId="0" xr:uid="{549490ED-661A-40A2-93ED-8A4235921A2E}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     kopie van AllergieIntolerantie GBB</t>
       </text>
     </comment>
     <comment ref="I13" authorId="1" shapeId="0" xr:uid="{13D6ADF7-ACBE-427D-B69D-85A079B82FC2}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     kopie van AllergieIntolerantie</t>
       </text>
     </comment>
     <comment ref="I15" authorId="2" shapeId="0" xr:uid="{2B12B02B-4733-400B-A2F6-75698B96C5E0}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     kopie van AllergieIntolerantie</t>
       </text>
     </comment>
     <comment ref="H26" authorId="3" shapeId="0" xr:uid="{E3DAE114-BFED-45BC-9D42-C0D3392F9B08}">
       <text>
-        <t>[Opmerkingenthread]
-U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
-Opmerking:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     als extensie wel</t>
       </text>
     </comment>
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="288">
   <si>
     <t>Veld</t>
   </si>
@@ -522,6 +522,12 @@
     <t>Vragen proeftuin</t>
   </si>
   <si>
+    <t>[Nummer van de informatie-requirement start bij 1, sub behoeftes kunnen worden gemodelleerd met X.X of X.X.X]</t>
+  </si>
+  <si>
+    <t>[Naam waaraan de informatie-requirement te herkennen is]</t>
+  </si>
+  <si>
     <t>[Geef hier een tekstuele omschrijving van de behoefte die ingevuld wordt met de informatie-requirement]</t>
   </si>
   <si>
@@ -531,10 +537,13 @@
     <t>[Geef aan in welke situaties het element waarmee de informatie-requirement gedekt wordt er zou moeten zijn, en evt. wanneer het afwezig kan zijn]</t>
   </si>
   <si>
+    <t>[Geef aan of de informatie relevant is voor gebruik van het model voor zaken in het verleden, in het heden, en/of de toekomst. Vaak is slechts een van deze situaties in scope van het bouwblok, maar niet altijd]</t>
+  </si>
+  <si>
     <t>[Geef aan waar de behoefte vandaan komt, bv. een specifieke informatiestandaard of bepaalde zorgrichtlijn]</t>
   </si>
   <si>
-    <t>EU-01</t>
+    <t>DEVICEUSE-01</t>
   </si>
   <si>
     <t xml:space="preserve">Status van het gebruik </t>
@@ -565,7 +574,7 @@
     <t>Nodig om te kunnen bepalen of het geregistreerde gebruik van het hulpmiddel actueel, beëindigd, gepland of anderszins niet actief is.</t>
   </si>
   <si>
-    <t>EU-02</t>
+    <t>DEVICEUSE-02</t>
   </si>
   <si>
     <t xml:space="preserve">De patiënt </t>
@@ -589,13 +598,33 @@
     <t>Nodig om het gebruik van het medische hulpmiddel ondubbelzinnig te relateren aan de patiënt die het hulpmiddel gebruikt, gebruikte of gaat gebruiken.</t>
   </si>
   <si>
+    <t>DEVICEUSE-03</t>
+  </si>
+  <si>
     <t>Informatie over het product dat gebruikt wordt als medisch hulpmiddel</t>
   </si>
   <si>
     <t>Geeft informatie over het medisch hulpmiddel die door de patiënt wordt gebruikt, gebruikt gaat worden of was gebruikt</t>
   </si>
   <si>
-    <t>EU-NL-03.01</t>
+    <t>String</t>
+  </si>
+  <si>
+    <t>Optioneel (0..1)</t>
+  </si>
+  <si>
+    <t>MedischHulpmiddel-v5.0(2024NL)
+MedischHulpmiddel-V3.3.1 (2020)
+MedischHulpmiddel-V3.1 (2017)</t>
+  </si>
+  <si>
+    <t>device.note (0..*)</t>
+  </si>
+  <si>
+    <t>Description (0..1)</t>
+  </si>
+  <si>
+    <t>DEVICEUSE-03.01</t>
   </si>
   <si>
     <t>Informatie over het medische hulpmiddel dat wordt gebruikt, zowel inwendig als uitwendig</t>
@@ -618,7 +647,7 @@
     <t>Nodig om vast te leggen welk medisch hulpmiddel door de patiënt wordt gebruikt. Zonder verwijzing naar het hulpmiddel kan de patiënt-hulpmiddelrelatie niet worden beschreven. Dit sluit ook aan bij de bestaande zib MedischHulpmiddel.</t>
   </si>
   <si>
-    <t>NL-03.02</t>
+    <t>DEVICEUSE-03.02</t>
   </si>
   <si>
     <t>Informatie van het type product dat gebruikt wordt als medisch hulpmiddel</t>
@@ -627,15 +656,7 @@
     <t>Het type product dat gebruikt wordt als medisch hulpmiddel</t>
   </si>
   <si>
-    <t>String of Codelijsten HIBRProductIDCodelijst, GTINProductIDCodelijst</t>
-  </si>
-  <si>
-    <t>Optioneel (0..1)</t>
-  </si>
-  <si>
-    <t>MedischHulpmiddel-v5.0(2024NL)
-MedischHulpmiddel-V3.3.1 (2020)
-MedischHulpmiddel-V3.1 (2017)</t>
+    <t>Codelijsten HIBRProductIDCodelijst, GTINProductIDCodelijst</t>
   </si>
   <si>
     <t>device.type (0..1)</t>
@@ -650,7 +671,19 @@
     <t xml:space="preserve">Is er naast de referentie naar Device nog informatie die onder dit element valt? Anders is een referentie naar Device voldoende. </t>
   </si>
   <si>
-    <t>NL-03.03</t>
+    <t>DEVICEUSE-03.03</t>
+  </si>
+  <si>
+    <t>Informatie van de product ID dat gebruikt wordt als medisch hulpmiddel</t>
+  </si>
+  <si>
+    <t>ID van het product dat gebruikt wordt als medisch hulpmiddel</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>DEVICEUSE-03.04</t>
   </si>
   <si>
     <r>
@@ -717,7 +750,7 @@
     <t>Wat doen we met dit element? Wordt ook besproken binnen Device</t>
   </si>
   <si>
-    <t>EU-04</t>
+    <t>DEVICEUSE-04</t>
   </si>
   <si>
     <t xml:space="preserve">Business identifier </t>
@@ -726,36 +759,39 @@
     <t>De behoefte aan een uniek, persistent business identifier</t>
   </si>
   <si>
-    <t>Identifier</t>
-  </si>
-  <si>
     <t>Optioneel (0..*)</t>
   </si>
   <si>
+    <t>EHDS logical model EDHSDeviceUse 1.0.0
+MedischHulpmiddel-v5.0(2024NL)
+MedischHulpmiddel-V3.3.1 (2020)
+MedischHulpmiddel-V3.1 (2017)</t>
+  </si>
+  <si>
+    <t>identifier (0..*)</t>
+  </si>
+  <si>
+    <t>ja maar komt niet voor in de archetypen, maar komt naar voren bij het opslaan (originating_system_item_ids : DV_IDENTIFIER). is 0..*</t>
+  </si>
+  <si>
+    <t>Nodig om een registratie van DeviceUse duurzaam en systeemoverstijgend te kunnen identificeren, zodat dezelfde registratie bij uitwisseling, verwerking en updates herkenbaar blijft.</t>
+  </si>
+  <si>
+    <t>DEVICEUSE-05</t>
+  </si>
+  <si>
+    <t>Auteur</t>
+  </si>
+  <si>
+    <t>Degene of hetgene welke de informatie over het concept heeft ingevuld</t>
+  </si>
+  <si>
+    <t>Referentie naar zorgverlener, zorgaanbieder of EHDSDevice</t>
+  </si>
+  <si>
     <t>EHDS logical model EDHSDeviceUse 1.0.0</t>
   </si>
   <si>
-    <t>identifier (0..*)</t>
-  </si>
-  <si>
-    <t>ja maar komt niet voor in de archetypen, maar komt naar voren bij het opslaan (originating_system_item_ids : DV_IDENTIFIER). is 0..*</t>
-  </si>
-  <si>
-    <t>Nodig om een registratie van DeviceUse duurzaam en systeemoverstijgend te kunnen identificeren, zodat dezelfde registratie bij uitwisseling, verwerking en updates herkenbaar blijft.</t>
-  </si>
-  <si>
-    <t>EU-05</t>
-  </si>
-  <si>
-    <t>Auteur</t>
-  </si>
-  <si>
-    <t>Degene of hetgene welke de informatie over het concept heeft ingevuld</t>
-  </si>
-  <si>
-    <t>Referentie naar zorgverlener, zorgaanbieder of EHDSDevice</t>
-  </si>
-  <si>
     <t>geen mapping</t>
   </si>
   <si>
@@ -765,7 +801,7 @@
     <t>Nodig wanneer herleidbaarheid vereist is van wie of wat de registratie over het gebruik heeft opgesteld. Heroverwegen of dit zorginhoudelijk onderdeel van DeviceUse moet zijn of generieke metadata/provenance.</t>
   </si>
   <si>
-    <t>EU-06</t>
+    <t>DEVICEUSE-06</t>
   </si>
   <si>
     <t xml:space="preserve">Moment van schrijven </t>
@@ -786,7 +822,7 @@
     <t>Nodig om te weten wanneer de registratie is vastgelegd. Heroverwegen als zib-element: dit beschrijft primair de registratie zelf en niet het klinische gebruik van het hulpmiddel en kan daarom mogelijk generiek als metadata/provenance worden opgelost.</t>
   </si>
   <si>
-    <t>EU-07</t>
+    <t>DEVICEUSE-07</t>
   </si>
   <si>
     <t>Bron van de informatie</t>
@@ -817,7 +853,7 @@
     <t>Nodig om de betrouwbaarheid en context van de informatie te kunnen beoordelen, bijvoorbeeld wanneer informatie door patiënt/vertegenwoordiger is aangeleverd.</t>
   </si>
   <si>
-    <t>EU-08</t>
+    <t>DEVICEUSE-08</t>
   </si>
   <si>
     <t>Gebruikte taal</t>
@@ -835,7 +871,7 @@
     <t>Nodig voor correcte verwerking van taalafhankelijke tekstuele gegevens bij grensoverschrijdende uitwisseling.</t>
   </si>
   <si>
-    <t>EU-09</t>
+    <t>DEVICEUSE-09</t>
   </si>
   <si>
     <t>Periode van gebruik</t>
@@ -856,7 +892,7 @@
     <t xml:space="preserve">Kunnen deze elementen worden samengevoegd? EHDS heeft een 'periode' met een start en eind datum. Binnen NL specificeren we een start en eind datum, geen periode. </t>
   </si>
   <si>
-    <t>NL-09.01</t>
+    <t>DEVICEUSE-09.01</t>
   </si>
   <si>
     <t>Startdatum van periode</t>
@@ -874,7 +910,7 @@
     <t>Nodig om te bepalen vanaf wanneer het hulpmiddel is toegepast of geïmplanteerd.</t>
   </si>
   <si>
-    <t>NL-09.02</t>
+    <t>DEVICEUSE-09.02</t>
   </si>
   <si>
     <t>Einddatum van periode</t>
@@ -896,7 +932,7 @@
     <t>Nodig om te bepalen wanneer gebruik of aanwezigheid van het hulpmiddel is beëindigd, bijvoorbeeld na explantatie.</t>
   </si>
   <si>
-    <t>EU-NL-10</t>
+    <t>DEVICEUSE-10</t>
   </si>
   <si>
     <t>Anatomische locatie</t>
@@ -908,7 +944,7 @@
     <t>Body site (0..1)</t>
   </si>
   <si>
-    <t>EU-NL-10.01</t>
+    <t>DEVICEUSE-10.01</t>
   </si>
   <si>
     <t>De behoefte om te verwijen naar de anatomische locatie. Anatomische locatie waarin het medische hulpmiddel zich bevindt. Dit kan ook lateraliteit bevatten</t>
@@ -928,7 +964,7 @@
     <t>Nodig wanneer de plaats van het hulpmiddel op/in het lichaam klinisch relevant is, bijvoorbeeld voor implantaten. Maakt het mogelijk te bepalen waar het hulpmiddel zich bevindt en eventueel aan welke zijde.</t>
   </si>
   <si>
-    <t>EU-NL-11</t>
+    <t>DEVICEUSE-11</t>
   </si>
   <si>
     <t xml:space="preserve">Reden van gebruik </t>
@@ -937,9 +973,6 @@
     <t>Reden of justificiatie van het gebruik van het medisch hulpmiddel</t>
   </si>
   <si>
-    <t>String</t>
-  </si>
-  <si>
     <t>reasonCode (0..*)</t>
   </si>
   <si>
@@ -949,7 +982,7 @@
     <t>Nodig om te begrijpen waarom de patiënt het hulpmiddel gebruikt. Dit geeft de klinische context voor de patiënt-hulpmiddelrelatie en maakt interpretatie mogelijk zonder de reden uit andere gegevens te hoeven afleiden.</t>
   </si>
   <si>
-    <t>EU-11.01</t>
+    <t>DEVICEUSE-11.01</t>
   </si>
   <si>
     <t>De behoefte om te kunnen verwijzen naar probleem, diagnose of procedure</t>
@@ -964,7 +997,7 @@
     <t>Hoe gaan we om met verwijzingen naar observation, condition, procedure etc</t>
   </si>
   <si>
-    <t>NL-11.02</t>
+    <t>DEVICEUSE-11.02</t>
   </si>
   <si>
     <t>De behoefte om te kunnen verwijzen naar de zib diagnose</t>
@@ -976,7 +1009,7 @@
     <t>MedischHulpmiddel-v5.0(2024NL)</t>
   </si>
   <si>
-    <t>NL-11.03</t>
+    <t>DEVICEUSE-11.03</t>
   </si>
   <si>
     <t>De behoefte om te kunnen verwijzen naar de zib probleem</t>
@@ -989,7 +1022,7 @@
 MedischHulpmiddel-V3.1 (2017)</t>
   </si>
   <si>
-    <t>EU-NL-12</t>
+    <t>DEVICEUSE-12</t>
   </si>
   <si>
     <t xml:space="preserve">Aanvullende informatie over het medisch hulpmiddeld die niet op een andere manier in het concept kan worden geduid. Dit kan ook informatie zijn over de toepassing van het medisch hulpmiddel  </t>
@@ -1003,13 +1036,10 @@
     <t>note (0..*)</t>
   </si>
   <si>
-    <t>Description (0..1)</t>
-  </si>
-  <si>
     <t>Nodig om relevante informatie over het gebruik of hulpmiddel vast te leggen die niet gestructureerd in de overige elementen kan worden uitgedrukt.</t>
   </si>
   <si>
-    <t>NL-13</t>
+    <t>DEVICEUSE-13</t>
   </si>
   <si>
     <t xml:space="preserve">Zorgverlener </t>
@@ -1030,7 +1060,7 @@
     <t xml:space="preserve">Zorgaanbieder versus auteur, beide relevant? Zo ja, toevoegen. Zo nee, uit informatiebehoefte halen. </t>
   </si>
   <si>
-    <t>NL-14</t>
+    <t>DEVICEUSE-14</t>
   </si>
   <si>
     <t>Zorgaanbieder als locatie</t>
@@ -1064,7 +1094,7 @@
   </si>
   <si>
     <t xml:space="preserve">
-In de zib MedischHulpmiddel zit de negetatie als codelijst ingebouwd. Er zijn al tickets van dat dit niet helemaal hoort. In de proeftuin samen bespreken dat dit wellicht meer een observation is. </t>
+In de zib MedischHulpmiddel zit de negatie als codelijst ingebouwd. Er zijn al tickets van dat dit niet helemaal hoort. In de proeftuin samen bespreken dat dit wellicht meer een observation is. </t>
   </si>
   <si>
     <t xml:space="preserve">De 'geen codelijst' nemen we niet mee in de GBB. </t>
@@ -1222,16 +1252,7 @@
     </r>
   </si>
   <si>
-    <t>Verwijzing naar probleem, diagnose of procedure</t>
-  </si>
-  <si>
-    <t>verwijzing naar zib diagnose</t>
-  </si>
-  <si>
-    <t>verwijzing naar zib probleem</t>
-  </si>
-  <si>
-    <t>verwijzing naar anatomisch locatie waarin het medische hulpmiddel zich bevindt.</t>
+    <t>2.16.840.1.113883.2.4.3.11.60.153.4.35/2026-08-20T00:00:00</t>
   </si>
 </sst>
 </file>
@@ -1352,7 +1373,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1385,31 +1406,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC00000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.749992370372631"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1453,7 +1450,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1493,6 +1490,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1526,6 +1526,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1549,6 +1552,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -1556,19 +1562,19 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1577,31 +1583,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
     <dxf>
@@ -2733,12 +2718,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="218.42578125" customWidth="1"/>
+    <col min="1" max="1" width="218.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3"/>
     </row>
   </sheetData>
@@ -2750,19 +2735,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="83.28515625" customWidth="1"/>
-    <col min="3" max="3" width="99.28515625" style="7" customWidth="1"/>
-    <col min="4" max="4" width="54.140625" customWidth="1"/>
+    <col min="2" max="2" width="83.33203125" customWidth="1"/>
+    <col min="3" max="3" width="99.33203125" style="7" customWidth="1"/>
+    <col min="4" max="4" width="54.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3"/>
       <c r="D1" s="7"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2774,7 +2759,7 @@
       </c>
       <c r="D2" s="7"/>
     </row>
-    <row r="3" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2786,12 +2771,12 @@
       </c>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B4" s="14"/>
       <c r="C4" s="12"/>
       <c r="D4" s="12"/>
     </row>
-    <row r="5" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2802,18 +2787,18 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="334.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="334.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="21" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>12</v>
       </c>
@@ -2824,7 +2809,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -2834,9 +2819,9 @@
       <c r="C8" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="21"/>
-    </row>
-    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="D8" s="22"/>
+    </row>
+    <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -2846,9 +2831,9 @@
       <c r="C9" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="22"/>
-    </row>
-    <row r="10" spans="1:4" ht="231" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D9" s="23"/>
+    </row>
+    <row r="10" spans="1:4" ht="231" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -2860,7 +2845,7 @@
       </c>
       <c r="D10" s="12"/>
     </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -2872,19 +2857,22 @@
       </c>
       <c r="D11" s="12"/>
     </row>
-    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>27</v>
       </c>
       <c r="B12" s="14" t="s">
         <v>28</v>
       </c>
+      <c r="C12" s="7" t="s">
+        <v>287</v>
+      </c>
       <c r="D12" s="7"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D13" s="7"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="D14" s="7"/>
     </row>
   </sheetData>
@@ -2900,18 +2888,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F46AB0B-2B50-43BB-B4AB-B029D8EBF054}">
   <dimension ref="A1:G25"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.42578125" style="5" customWidth="1"/>
+    <col min="1" max="1" width="28.44140625" style="5" customWidth="1"/>
     <col min="2" max="2" width="40" style="4" customWidth="1"/>
-    <col min="3" max="3" width="51.42578125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="39.7109375" style="5" customWidth="1"/>
-    <col min="5" max="5" width="49.5703125" style="4" customWidth="1"/>
-    <col min="6" max="6" width="61.42578125" style="5" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="4"/>
+    <col min="3" max="3" width="51.44140625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="39.6640625" style="5" customWidth="1"/>
+    <col min="5" max="5" width="49.5546875" style="4" customWidth="1"/>
+    <col min="6" max="6" width="61.44140625" style="5" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>29</v>
       </c>
@@ -2932,7 +2920,7 @@
       </c>
       <c r="G1" s="5"/>
     </row>
-    <row r="2" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>35</v>
       </c>
@@ -2945,11 +2933,11 @@
       <c r="D2" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="20" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>35</v>
       </c>
@@ -2962,11 +2950,11 @@
       <c r="D3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="16" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>35</v>
       </c>
@@ -2979,25 +2967,25 @@
       <c r="D4" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="16" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="24" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="23" t="s">
+    <row r="5" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="F5" s="25" t="s">
+      <c r="F5" s="26" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>47</v>
       </c>
@@ -3007,11 +2995,11 @@
       <c r="D6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="16" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>47</v>
       </c>
@@ -3024,11 +3012,11 @@
       <c r="D7" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="16" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>47</v>
       </c>
@@ -3041,11 +3029,11 @@
       <c r="D8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="16" t="s">
+      <c r="F8" s="17" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>59</v>
       </c>
@@ -3055,11 +3043,11 @@
       <c r="C9" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="16" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>63</v>
       </c>
@@ -3072,11 +3060,11 @@
       <c r="D10" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="16" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>63</v>
       </c>
@@ -3089,11 +3077,11 @@
       <c r="D11" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="16" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>59</v>
       </c>
@@ -3103,11 +3091,11 @@
       <c r="C12" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F12" s="15" t="s">
+      <c r="F12" s="16" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>63</v>
       </c>
@@ -3117,11 +3105,11 @@
       <c r="C13" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="16" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>59</v>
       </c>
@@ -3131,11 +3119,11 @@
       <c r="C14" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="F14" s="16" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>63</v>
       </c>
@@ -3146,7 +3134,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>59</v>
       </c>
@@ -3157,7 +3145,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>59</v>
       </c>
@@ -3168,7 +3156,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>59</v>
       </c>
@@ -3179,7 +3167,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>59</v>
       </c>
@@ -3190,7 +3178,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>59</v>
       </c>
@@ -3201,7 +3189,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>59</v>
       </c>
@@ -3212,7 +3200,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>63</v>
       </c>
@@ -3223,7 +3211,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>59</v>
       </c>
@@ -3234,7 +3222,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>59</v>
       </c>
@@ -3245,7 +3233,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>59</v>
       </c>
@@ -3282,793 +3270,848 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
   <dimension ref="A1:K35"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.85546875" style="45" customWidth="1"/>
-    <col min="2" max="2" width="45.5703125" style="7" customWidth="1"/>
-    <col min="3" max="3" width="90.85546875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="52.140625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="28.7109375" style="27" customWidth="1"/>
-    <col min="6" max="6" width="28.7109375" style="7" customWidth="1"/>
-    <col min="7" max="7" width="48.7109375" style="27" customWidth="1"/>
+    <col min="1" max="1" width="19.88671875" style="28" customWidth="1"/>
+    <col min="2" max="2" width="45.5546875" style="7" customWidth="1"/>
+    <col min="3" max="3" width="90.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="52.109375" style="7" customWidth="1"/>
+    <col min="5" max="5" width="28.6640625" style="29" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="48.6640625" style="29" customWidth="1"/>
     <col min="8" max="8" width="25" style="7" customWidth="1"/>
     <col min="9" max="9" width="47" style="7" customWidth="1"/>
-    <col min="10" max="10" width="77.7109375" style="7" customWidth="1"/>
-    <col min="11" max="11" width="58.85546875" style="7" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="27"/>
+    <col min="10" max="10" width="77.6640625" style="7" customWidth="1"/>
+    <col min="11" max="11" width="58.88671875" style="7" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:11" s="29" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="46" t="s">
+    <row r="1" spans="1:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:11" s="31" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="30" t="s">
         <v>88</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="30" t="s">
         <v>89</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="30" t="s">
         <v>91</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="G2" s="28" t="s">
+      <c r="G2" s="30" t="s">
         <v>93</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="I2" s="28" t="s">
+      <c r="I2" s="30" t="s">
         <v>95</v>
       </c>
-      <c r="J2" s="36" t="s">
+      <c r="J2" s="39" t="s">
         <v>96</v>
       </c>
-      <c r="K2" s="36" t="s">
+      <c r="K2" s="39" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="141.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="47"/>
-      <c r="B3" s="26"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-    </row>
-    <row r="5" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="45" t="s">
+    <row r="3" spans="1:11" ht="141.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="F3" s="6" t="s">
         <v>103</v>
       </c>
+      <c r="G3" s="6" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E4" s="29" t="s">
+        <v>109</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="H4" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="I4" s="34" t="s">
+        <v>113</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>116</v>
+      </c>
       <c r="C5" s="5" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="E5" s="27" t="s">
-        <v>106</v>
+        <v>118</v>
+      </c>
+      <c r="E5" s="29" t="s">
+        <v>109</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="H5" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="H5" s="33" t="s">
+        <v>120</v>
+      </c>
+      <c r="I5" s="33" t="s">
+        <v>121</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A6" s="28" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E6" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="H6" s="33" t="s">
+        <v>129</v>
+      </c>
+      <c r="I6" s="33" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="60.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E7" s="29" t="s">
         <v>109</v>
       </c>
-      <c r="I5" s="32" t="s">
+      <c r="F7" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="H7" s="33" t="s">
+        <v>135</v>
+      </c>
+      <c r="I7" s="33" t="s">
+        <v>136</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="28" t="s">
+        <v>138</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>139</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="H8" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="I8" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="28" t="s">
+        <v>146</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>147</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="E9" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="H9" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="I9" s="34" t="s">
+        <v>143</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A10" s="28" t="s">
+        <v>150</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E10" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="J5" s="7" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="45" t="s">
-        <v>112</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>113</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="E6" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="H6" s="31" t="s">
-        <v>117</v>
-      </c>
-      <c r="I6" s="31" t="s">
-        <v>118</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="45">
-        <v>3</v>
-      </c>
-      <c r="B7" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="45" t="s">
-        <v>122</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>120</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="E8" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="H8" s="31" t="s">
-        <v>126</v>
-      </c>
-      <c r="I8" s="31" t="s">
-        <v>127</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="48" t="s">
-        <v>129</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>130</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="E9" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="H9" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="I9" s="32" t="s">
-        <v>136</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="49" t="s">
-        <v>139</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>140</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>141</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="G10" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="H10" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="E10" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="G10" s="7" t="s">
+      <c r="I10" s="34" t="s">
         <v>143</v>
       </c>
-      <c r="H10" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="I10" s="32" t="s">
-        <v>136</v>
-      </c>
       <c r="J10" s="3" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="45" t="s">
-        <v>146</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>147</v>
+        <v>156</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="59.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="28" t="s">
+        <v>157</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>158</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="E11" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="F11" s="37" t="s">
-        <v>116</v>
+      <c r="E11" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="F11" s="40" t="s">
+        <v>119</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="H11" s="31" t="s">
-        <v>152</v>
-      </c>
-      <c r="I11" s="33" t="s">
-        <v>153</v>
+        <v>161</v>
+      </c>
+      <c r="H11" s="33" t="s">
+        <v>162</v>
+      </c>
+      <c r="I11" s="35" t="s">
+        <v>163</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A12" s="45" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>156</v>
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="28" t="s">
+        <v>165</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>166</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="E12" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="F12" s="37" t="s">
-        <v>116</v>
+        <v>168</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="F12" s="40" t="s">
+        <v>119</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="H12" s="34" t="s">
-        <v>159</v>
-      </c>
-      <c r="I12" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="H12" s="36" t="s">
+        <v>170</v>
+      </c>
+      <c r="I12" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="J12" s="13" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A13" s="28" t="s">
+        <v>173</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="E13" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F13" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="H13" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="I13" s="35" t="s">
+        <v>178</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="28" t="s">
+        <v>180</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>181</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="E14" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F14" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="H14" s="33" t="s">
+        <v>184</v>
+      </c>
+      <c r="I14" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="28" t="s">
+        <v>186</v>
+      </c>
+      <c r="B15" s="18" t="s">
+        <v>187</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="E15" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F15" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="H15" s="33" t="s">
+        <v>190</v>
+      </c>
+      <c r="I15" s="35" t="s">
+        <v>178</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="B16" s="18" t="s">
+        <v>193</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="E16" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F16" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="H16" s="33" t="s">
+        <v>196</v>
+      </c>
+      <c r="I16" s="33"/>
+      <c r="J16" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="K16" s="47" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" s="43" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="28" t="s">
+        <v>199</v>
+      </c>
+      <c r="B17" s="41" t="s">
+        <v>200</v>
+      </c>
+      <c r="C17" s="41" t="s">
+        <v>201</v>
+      </c>
+      <c r="D17" s="42" t="s">
+        <v>176</v>
+      </c>
+      <c r="E17" s="43" t="s">
+        <v>127</v>
+      </c>
+      <c r="F17" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="G17" s="41" t="s">
+        <v>128</v>
+      </c>
+      <c r="H17" s="42" t="s">
+        <v>202</v>
+      </c>
+      <c r="I17" s="42" t="s">
+        <v>203</v>
+      </c>
+      <c r="J17" s="42" t="s">
+        <v>204</v>
+      </c>
+      <c r="K17" s="47"/>
+    </row>
+    <row r="18" spans="1:11" s="43" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="28" t="s">
+        <v>205</v>
+      </c>
+      <c r="B18" s="41" t="s">
+        <v>206</v>
+      </c>
+      <c r="C18" s="41" t="s">
+        <v>207</v>
+      </c>
+      <c r="D18" s="42" t="s">
+        <v>176</v>
+      </c>
+      <c r="E18" s="43" t="s">
+        <v>127</v>
+      </c>
+      <c r="F18" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="G18" s="41" t="s">
+        <v>208</v>
+      </c>
+      <c r="H18" s="42" t="s">
+        <v>209</v>
+      </c>
+      <c r="I18" s="42" t="s">
+        <v>210</v>
+      </c>
+      <c r="J18" s="45" t="s">
+        <v>211</v>
+      </c>
+      <c r="K18" s="47"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="28" t="s">
+        <v>212</v>
+      </c>
+      <c r="B19" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="F19" s="40"/>
+      <c r="H19" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="I19" s="33" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="28" t="s">
+        <v>216</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="E20" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F20" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="H20" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="I20" s="33" t="s">
+        <v>220</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="28" t="s">
+        <v>222</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E21" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F21" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="H21" s="33" t="s">
+        <v>225</v>
+      </c>
+      <c r="I21" s="36" t="s">
+        <v>226</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="B22" s="18"/>
+      <c r="C22" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="E22" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="J12" s="13" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="60" x14ac:dyDescent="0.25">
-      <c r="A13" s="45" t="s">
-        <v>162</v>
-      </c>
-      <c r="B13" s="17" t="s">
-        <v>163</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="E13" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F13" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="H13" s="31" t="s">
-        <v>166</v>
-      </c>
-      <c r="I13" s="33" t="s">
-        <v>167</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="45" t="s">
+      <c r="F22" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G22" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>170</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="H22" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="I22" s="36"/>
+      <c r="K22" s="47" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="28" t="s">
+        <v>233</v>
+      </c>
+      <c r="B23" s="18"/>
+      <c r="C23" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="E23" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="F23" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="H23" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="I23" s="36"/>
+      <c r="K23" s="47"/>
+    </row>
+    <row r="24" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="28" t="s">
+        <v>237</v>
+      </c>
+      <c r="B24" s="18"/>
+      <c r="C24" s="38" t="s">
+        <v>238</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="E24" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="F24" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="H24" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="I24" s="36"/>
+      <c r="K24" s="47"/>
+    </row>
+    <row r="25" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="28" t="s">
+        <v>241</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E25" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F25" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>243</v>
+      </c>
+      <c r="H25" s="33" t="s">
+        <v>244</v>
+      </c>
+      <c r="I25" s="33" t="s">
+        <v>130</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>247</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="E26" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F26" s="40" t="s">
+        <v>119</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="H26" s="36" t="s">
+        <v>250</v>
+      </c>
+      <c r="I26" s="33" t="s">
         <v>171</v>
       </c>
-      <c r="D14" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="E14" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F14" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="H14" s="31" t="s">
-        <v>173</v>
-      </c>
-      <c r="I14" s="31" t="s">
-        <v>160</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="45" t="s">
-        <v>175</v>
-      </c>
-      <c r="B15" s="17" t="s">
-        <v>176</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="D15" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F15" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="H15" s="31" t="s">
-        <v>179</v>
-      </c>
-      <c r="I15" s="33" t="s">
-        <v>167</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="50" t="s">
-        <v>181</v>
-      </c>
-      <c r="B16" s="17" t="s">
-        <v>182</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F16" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="H16" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="I16" s="31"/>
-      <c r="J16" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="K16" s="44" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" s="40" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A17" s="50" t="s">
-        <v>188</v>
-      </c>
-      <c r="B17" s="38" t="s">
-        <v>189</v>
-      </c>
-      <c r="C17" s="38" t="s">
-        <v>190</v>
-      </c>
-      <c r="D17" s="39" t="s">
-        <v>165</v>
-      </c>
-      <c r="E17" s="40" t="s">
-        <v>133</v>
-      </c>
-      <c r="F17" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>134</v>
-      </c>
-      <c r="H17" s="39" t="s">
-        <v>191</v>
-      </c>
-      <c r="I17" s="39" t="s">
-        <v>192</v>
-      </c>
-      <c r="J17" s="39" t="s">
-        <v>193</v>
-      </c>
-      <c r="K17" s="44"/>
-    </row>
-    <row r="18" spans="1:11" s="40" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="50" t="s">
-        <v>194</v>
-      </c>
-      <c r="B18" s="38" t="s">
-        <v>195</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>196</v>
-      </c>
-      <c r="D18" s="39" t="s">
-        <v>165</v>
-      </c>
-      <c r="E18" s="40" t="s">
-        <v>133</v>
-      </c>
-      <c r="F18" s="41" t="s">
-        <v>116</v>
-      </c>
-      <c r="G18" s="38" t="s">
-        <v>197</v>
-      </c>
-      <c r="H18" s="39" t="s">
-        <v>198</v>
-      </c>
-      <c r="I18" s="39" t="s">
-        <v>199</v>
-      </c>
-      <c r="J18" s="42" t="s">
-        <v>200</v>
-      </c>
-      <c r="K18" s="44"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="45" t="s">
-        <v>201</v>
-      </c>
-      <c r="B19" s="17" t="s">
-        <v>202</v>
-      </c>
-      <c r="F19" s="37"/>
-      <c r="H19" s="31" t="s">
-        <v>203</v>
-      </c>
-      <c r="I19" s="31" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A20" s="45" t="s">
-        <v>205</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>281</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="E20" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F20" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>208</v>
-      </c>
-      <c r="H20" s="31" t="s">
-        <v>203</v>
-      </c>
-      <c r="I20" s="31" t="s">
-        <v>209</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="45" t="s">
-        <v>211</v>
-      </c>
-      <c r="B21" s="17" t="s">
-        <v>212</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="E21" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F21" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="H21" s="31" t="s">
-        <v>215</v>
-      </c>
-      <c r="I21" s="34" t="s">
-        <v>216</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="45" t="s">
-        <v>218</v>
-      </c>
-      <c r="B22" s="17" t="s">
-        <v>278</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="E22" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="F22" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G22" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="H22" s="31" t="s">
-        <v>221</v>
-      </c>
-      <c r="I22" s="34"/>
-      <c r="K22" s="44" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="45" t="s">
-        <v>223</v>
-      </c>
-      <c r="B23" s="17" t="s">
-        <v>279</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>224</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="E23" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="F23" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="H23" s="31" t="s">
-        <v>221</v>
-      </c>
-      <c r="I23" s="34"/>
-      <c r="K23" s="44"/>
-    </row>
-    <row r="24" spans="1:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="45" t="s">
-        <v>227</v>
-      </c>
-      <c r="B24" s="17" t="s">
-        <v>280</v>
-      </c>
-      <c r="C24" s="35" t="s">
-        <v>228</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="E24" s="27" t="s">
-        <v>150</v>
-      </c>
-      <c r="F24" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G24" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="H24" s="31" t="s">
-        <v>221</v>
-      </c>
-      <c r="I24" s="34"/>
-      <c r="K24" s="44"/>
-    </row>
-    <row r="25" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A25" s="45" t="s">
-        <v>231</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>214</v>
-      </c>
-      <c r="E25" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F25" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="H25" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="I25" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A26" s="51" t="s">
-        <v>237</v>
-      </c>
-      <c r="B26" s="17" t="s">
-        <v>238</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="E26" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F26" s="37" t="s">
-        <v>116</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="H26" s="34" t="s">
-        <v>241</v>
-      </c>
-      <c r="I26" s="31" t="s">
-        <v>160</v>
-      </c>
       <c r="J26" s="3" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A27" s="51" t="s">
-        <v>244</v>
-      </c>
-      <c r="B27" s="17" t="s">
-        <v>245</v>
+        <v>252</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="28" t="s">
+        <v>253</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>254</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>247</v>
-      </c>
-      <c r="E27" s="27" t="s">
-        <v>133</v>
-      </c>
-      <c r="F27" s="37" t="s">
-        <v>116</v>
+        <v>256</v>
+      </c>
+      <c r="E27" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="F27" s="40" t="s">
+        <v>119</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="H27" s="34" t="s">
-        <v>241</v>
-      </c>
-      <c r="I27" s="31" t="s">
-        <v>160</v>
+        <v>128</v>
+      </c>
+      <c r="H27" s="36" t="s">
+        <v>250</v>
+      </c>
+      <c r="I27" s="33" t="s">
+        <v>171</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="K27" s="7" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B28" s="17"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B29" s="17"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B30" s="17"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B31" s="17"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B32" s="17"/>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B33" s="17"/>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B34" s="17"/>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B35" s="17"/>
+        <v>258</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B28" s="18"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B29" s="18"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B30" s="18"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B31" s="18"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B32" s="18"/>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B33" s="18"/>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B34" s="18"/>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B35" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4085,94 +4128,94 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B424468-1DFA-48A4-A0AA-9F487915F6EF}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="27"/>
-    <col min="2" max="2" width="40.5703125" style="27" customWidth="1"/>
-    <col min="3" max="3" width="83.42578125" style="27" customWidth="1"/>
-    <col min="4" max="4" width="32.42578125" style="7" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="27"/>
+    <col min="1" max="1" width="9.109375" style="29"/>
+    <col min="2" max="2" width="40.5546875" style="29" customWidth="1"/>
+    <col min="3" max="3" width="83.44140625" style="29" customWidth="1"/>
+    <col min="4" max="4" width="32.44140625" style="7" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="29"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
-        <v>250</v>
-      </c>
-      <c r="B1" s="27" t="s">
-        <v>251</v>
-      </c>
-      <c r="C1" s="27" t="s">
-        <v>252</v>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="29" t="s">
+        <v>259</v>
+      </c>
+      <c r="B1" s="29" t="s">
+        <v>260</v>
+      </c>
+      <c r="C1" s="29" t="s">
+        <v>261</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="43">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="46">
         <v>46247</v>
       </c>
-      <c r="B2" s="27" t="s">
-        <v>254</v>
+      <c r="B2" s="29" t="s">
+        <v>263</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="43">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="46">
         <v>46247</v>
       </c>
-      <c r="B3" s="27" t="s">
-        <v>257</v>
+      <c r="B3" s="29" t="s">
+        <v>266</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="270" x14ac:dyDescent="0.25">
-      <c r="A4" s="43">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="244.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="46">
         <v>46247</v>
       </c>
-      <c r="B4" s="27" t="s">
-        <v>260</v>
+      <c r="B4" s="29" t="s">
+        <v>269</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="43">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="46">
         <v>46247</v>
       </c>
-      <c r="B5" s="27" t="s">
-        <v>263</v>
-      </c>
-      <c r="C5" s="27" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="225" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="43">
+      <c r="B5" s="29" t="s">
+        <v>272</v>
+      </c>
+      <c r="C5" s="29" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="225" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="46">
         <v>46247</v>
       </c>
-      <c r="B6" s="27" t="s">
-        <v>265</v>
+      <c r="B6" s="29" t="s">
+        <v>274</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -4183,22 +4226,22 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" customWidth="1"/>
-    <col min="2" max="2" width="18.5703125" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" customWidth="1"/>
-    <col min="7" max="7" width="41.5703125" customWidth="1"/>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" customWidth="1"/>
+    <col min="7" max="7" width="41.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>88</v>
@@ -4216,27 +4259,27 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -4248,9 +4291,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" ht="111" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1" ht="111" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -4260,37 +4303,37 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11888EB5-97B2-4D4F-80A1-6855BF5D9AE8}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" customWidth="1"/>
-    <col min="2" max="2" width="92.28515625" customWidth="1"/>
+    <col min="1" max="1" width="37.44140625" customWidth="1"/>
+    <col min="2" max="2" width="92.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="177.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="177.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>272</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+        <v>281</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="171" customHeight="1" x14ac:dyDescent="0.25">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="171" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="B3" s="18" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>285</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B8" s="4"/>
       <c r="C8" s="5"/>
       <c r="D8" s="4"/>
@@ -4303,6 +4346,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -4509,17 +4563,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -4530,6 +4573,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4548,17 +4602,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
DeviceUse: excel file refresh
</commit_message>
<xml_diff>
--- a/input/requirements/DeviceUse.xlsx
+++ b/input/requirements/DeviceUse.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MichalCiszewski\Documents\Github\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62246BE6-3BA6-4081-A4F7-0E4AB2677F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E873502A-EC35-43DA-9917-5EA8F879914C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="2" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -48,7 +48,7 @@
     <author>tc={34562484-290B-4F2D-9790-FE82BD1E616C}</author>
   </authors>
   <commentList>
-    <comment ref="C10" authorId="0" shapeId="0" xr:uid="{34562484-290B-4F2D-9790-FE82BD1E616C}">
+    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{34562484-290B-4F2D-9790-FE82BD1E616C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -71,7 +71,7 @@
     <author>tc={E3DAE114-BFED-45BC-9D42-C0D3392F9B08}</author>
   </authors>
   <commentList>
-    <comment ref="I11" authorId="0" shapeId="0" xr:uid="{549490ED-661A-40A2-93ED-8A4235921A2E}">
+    <comment ref="I10" authorId="0" shapeId="0" xr:uid="{549490ED-661A-40A2-93ED-8A4235921A2E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -79,7 +79,7 @@
     kopie van AllergieIntolerantie GBB</t>
       </text>
     </comment>
-    <comment ref="I13" authorId="1" shapeId="0" xr:uid="{13D6ADF7-ACBE-427D-B69D-85A079B82FC2}">
+    <comment ref="I12" authorId="1" shapeId="0" xr:uid="{13D6ADF7-ACBE-427D-B69D-85A079B82FC2}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -87,7 +87,7 @@
     kopie van AllergieIntolerantie</t>
       </text>
     </comment>
-    <comment ref="I15" authorId="2" shapeId="0" xr:uid="{2B12B02B-4733-400B-A2F6-75698B96C5E0}">
+    <comment ref="I14" authorId="2" shapeId="0" xr:uid="{2B12B02B-4733-400B-A2F6-75698B96C5E0}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +95,7 @@
     kopie van AllergieIntolerantie</t>
       </text>
     </comment>
-    <comment ref="H26" authorId="3" shapeId="0" xr:uid="{E3DAE114-BFED-45BC-9D42-C0D3392F9B08}">
+    <comment ref="H25" authorId="3" shapeId="0" xr:uid="{E3DAE114-BFED-45BC-9D42-C0D3392F9B08}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="275">
   <si>
     <t>Veld</t>
   </si>
@@ -116,13 +116,7 @@
     <t>Beschrijving</t>
   </si>
   <si>
-    <t>Invulling van het veld</t>
-  </si>
-  <si>
     <t>Conceptbeschrijving</t>
-  </si>
-  <si>
-    <t>[De definitie of beschrijving van het concept.]</t>
   </si>
   <si>
     <r>
@@ -177,9 +171,6 @@
     <t>Doel</t>
   </si>
   <si>
-    <t>[De doelen en redenen om het concept vast te leggen en/of uit te wisselen.]</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -211,9 +202,6 @@
   </si>
   <si>
     <t>Gebruiksscenario(’s)</t>
-  </si>
-  <si>
-    <t>[Geeft aan in welke context(en) het concept wordt gebruikt. Geef voorbeelden van gebruik in informatiestandaarden.]</t>
   </si>
   <si>
     <r>
@@ -260,25 +248,16 @@
     <t>Representatie</t>
   </si>
   <si>
-    <t>[Beschrijf hier wat er voor de dossiervorming belangrijk is rondom de levenscyclus en instantiaties van het concept.]</t>
-  </si>
-  <si>
     <t>Informatie over een medisch hulpmiddel van een patiënt kan in de loop van de tijd veranderen. Het heeft onder andere een begin en een einddatum. Daarnaast kan de toelichting over het medische hulpmiddel ook aangepast worden over de tijd. Ook de anatomische locatie kan eventueel wijzigen. En de reden is optioneel.</t>
   </si>
   <si>
     <t>Alias(sen)</t>
   </si>
   <si>
-    <t>[Alle bekende synoniemen voor het concept.]</t>
-  </si>
-  <si>
     <t xml:space="preserve">Implantaat; apparatuur; uitwendige apparatuur; (patiëntgebonden) hulpmiddel; </t>
   </si>
   <si>
     <t>Juist gebruik</t>
-  </si>
-  <si>
-    <t>[Beschrijf hier waarvoor het concept wél bedoeld is].</t>
   </si>
   <si>
     <t xml:space="preserve">Het concept is bedoeld om het gebruik van het medsich hulpmiddel dat op/in een patiënt zit uit te wisselen. 
@@ -286,9 +265,6 @@
   </si>
   <si>
     <t>Onjuist gebruik</t>
-  </si>
-  <si>
-    <t>[Beschrijf hier waar het concept niet voor bedoeld is, en geef waar mogelijk aan welk concept er wel geschikt voor is.]</t>
   </si>
   <si>
     <t>Het is niet bedoeld om dit concept te gebruiken als auteur of registrator van de gegevens. 
@@ -302,16 +278,10 @@
     <t>Referenties</t>
   </si>
   <si>
-    <t>[Relevante bronstandaarden of informatiebronnen die het ontwerp en de scope van het concept hebben beïnvloed.]</t>
-  </si>
-  <si>
     <t>Zie tabblad 'bronnen'</t>
   </si>
   <si>
     <t>ART-DECOR-id</t>
-  </si>
-  <si>
-    <t>[Het id op ART-DECOR van het afsprakenmodel, bv 2.16.840.1.113883.2.4.3.11.60.153.4.12/2026-06-04T00:00:00]</t>
   </si>
   <si>
     <t>Type bron</t>
@@ -522,12 +492,6 @@
     <t>Vragen proeftuin</t>
   </si>
   <si>
-    <t>[Nummer van de informatie-requirement start bij 1, sub behoeftes kunnen worden gemodelleerd met X.X of X.X.X]</t>
-  </si>
-  <si>
-    <t>[Naam waaraan de informatie-requirement te herkennen is]</t>
-  </si>
-  <si>
     <t>[Geef hier een tekstuele omschrijving van de behoefte die ingevuld wordt met de informatie-requirement]</t>
   </si>
   <si>
@@ -535,9 +499,6 @@
   </si>
   <si>
     <t>[Geef aan in welke situaties het element waarmee de informatie-requirement gedekt wordt er zou moeten zijn, en evt. wanneer het afwezig kan zijn]</t>
-  </si>
-  <si>
-    <t>[Geef aan of de informatie relevant is voor gebruik van het model voor zaken in het verleden, in het heden, en/of de toekomst. Vaak is slechts een van deze situaties in scope van het bouwblok, maar niet altijd]</t>
   </si>
   <si>
     <t>[Geef aan waar de behoefte vandaan komt, bv. een specifieke informatiestandaard of bepaalde zorgrichtlijn]</t>
@@ -1259,7 +1220,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1282,13 +1243,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -1448,9 +1402,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1463,13 +1417,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1481,50 +1432,41 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -1537,7 +1479,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1555,14 +1497,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1571,7 +1513,7 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1588,7 +1530,7 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="9">
     <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1615,25 +1557,6 @@
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1766,7 +1689,7 @@
       <xdr:rowOff>223837</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>342900</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>2181225</xdr:rowOff>
@@ -2346,12 +2269,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96E5C6F6-FD6C-477B-B67D-E91A0233B27C}" name="Tabel1" displayName="Tabel1" ref="A2:C12" totalsRowShown="0">
-  <autoFilter ref="A2:C12" xr:uid="{96E5C6F6-FD6C-477B-B67D-E91A0233B27C}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96E5C6F6-FD6C-477B-B67D-E91A0233B27C}" name="Tabel1" displayName="Tabel1" ref="A2:B12" totalsRowShown="0">
+  <autoFilter ref="A2:B12" xr:uid="{96E5C6F6-FD6C-477B-B67D-E91A0233B27C}"/>
+  <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{37EF08FA-B565-414A-A476-BC12FA6A1A1B}" name="Veld"/>
-    <tableColumn id="2" xr3:uid="{E6708E34-04D9-4C68-AE5D-AA79CB057466}" name="Beschrijving" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{DDB6E257-D214-4298-B27F-676B3675AD2B}" name="Invulling van het veld" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{DDB6E257-D214-4298-B27F-676B3675AD2B}" name="Beschrijving" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2689,10 +2611,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C10" dT="2026-07-09T09:29:17.34" personId="{7313A655-1F36-4FD7-A150-7E7D12B2EDEE}" id="{34562484-290B-4F2D-9790-FE82BD1E616C}" done="1">
+  <threadedComment ref="B10" dT="2026-07-09T09:29:17.34" personId="{7313A655-1F36-4FD7-A150-7E7D12B2EDEE}" id="{34562484-290B-4F2D-9790-FE82BD1E616C}" done="1">
     <text>Of, is dit concept wel bedoelt voor aanlevering LIR? Het zou wel kunnen, maar dan hebben we het over een andere use case dan zorg-zorg. We hebben het dan over zorg-overheid. bestaat zon use case al?</text>
   </threadedComment>
-  <threadedComment ref="C10" dT="2026-07-20T09:49:23.46" personId="{1A9903B1-95BB-4B80-8FB6-9CB6AE3DAE32}" id="{46A8CD43-C164-44C4-9E7B-D71ECE1B481A}" parentId="{34562484-290B-4F2D-9790-FE82BD1E616C}">
+  <threadedComment ref="B10" dT="2026-07-20T09:49:23.46" personId="{1A9903B1-95BB-4B80-8FB6-9CB6AE3DAE32}" id="{46A8CD43-C164-44C4-9E7B-D71ECE1B481A}" parentId="{34562484-290B-4F2D-9790-FE82BD1E616C}">
     <text>Zowel de bouwblokken Device als DeviceUse zijn nodig voor LIR</text>
   </threadedComment>
 </ThreadedComments>
@@ -2700,16 +2622,16 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="I11" dT="2026-07-10T14:04:40.43" personId="{2433C95E-497B-4508-8AFD-092CFDE71E25}" id="{549490ED-661A-40A2-93ED-8A4235921A2E}">
+  <threadedComment ref="I10" dT="2026-07-10T14:04:40.43" personId="{2433C95E-497B-4508-8AFD-092CFDE71E25}" id="{549490ED-661A-40A2-93ED-8A4235921A2E}">
     <text>kopie van AllergieIntolerantie GBB</text>
   </threadedComment>
-  <threadedComment ref="I13" dT="2026-07-10T14:04:45.56" personId="{2433C95E-497B-4508-8AFD-092CFDE71E25}" id="{13D6ADF7-ACBE-427D-B69D-85A079B82FC2}">
+  <threadedComment ref="I12" dT="2026-07-10T14:04:45.56" personId="{2433C95E-497B-4508-8AFD-092CFDE71E25}" id="{13D6ADF7-ACBE-427D-B69D-85A079B82FC2}">
     <text>kopie van AllergieIntolerantie</text>
   </threadedComment>
-  <threadedComment ref="I15" dT="2026-07-10T14:04:45.56" personId="{2433C95E-497B-4508-8AFD-092CFDE71E25}" id="{2B12B02B-4733-400B-A2F6-75698B96C5E0}">
+  <threadedComment ref="I14" dT="2026-07-10T14:04:45.56" personId="{2433C95E-497B-4508-8AFD-092CFDE71E25}" id="{2B12B02B-4733-400B-A2F6-75698B96C5E0}">
     <text>kopie van AllergieIntolerantie</text>
   </threadedComment>
-  <threadedComment ref="H26" dT="2026-07-10T14:17:42.01" personId="{2433C95E-497B-4508-8AFD-092CFDE71E25}" id="{E3DAE114-BFED-45BC-9D42-C0D3392F9B08}">
+  <threadedComment ref="H25" dT="2026-07-10T14:17:42.01" personId="{2433C95E-497B-4508-8AFD-092CFDE71E25}" id="{E3DAE114-BFED-45BC-9D42-C0D3392F9B08}">
     <text>als extensie wel</text>
   </threadedComment>
 </ThreadedComments>
@@ -2734,146 +2656,114 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="83.33203125" customWidth="1"/>
-    <col min="3" max="3" width="99.33203125" style="7" customWidth="1"/>
-    <col min="4" max="4" width="54.109375" customWidth="1"/>
+    <col min="2" max="2" width="99.33203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="54.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3"/>
-      <c r="D1" s="7"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C1" s="6"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6"/>
+    </row>
+    <row r="3" spans="1:3" ht="78.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="7"/>
-    </row>
-    <row r="3" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="B3" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="12"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="B4" s="11"/>
+      <c r="C4" s="11"/>
+    </row>
+    <row r="5" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="B5" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B4" s="14"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-    </row>
-    <row r="5" spans="1:4" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="334.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B6" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="13" t="s">
+    </row>
+    <row r="7" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="334.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="B7" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="14" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="B8" s="6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="C8" s="19"/>
+    </row>
+    <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B9" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C9" s="20"/>
+    </row>
+    <row r="10" spans="1:3" ht="231" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B10" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="C10" s="11"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="22"/>
-    </row>
-    <row r="9" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="C11" s="11"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="23"/>
-    </row>
-    <row r="10" spans="1:4" ht="231" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="12"/>
-    </row>
-    <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="12"/>
-    </row>
-    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>287</v>
-      </c>
-      <c r="D12" s="7"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D13" s="7"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="D14" s="7"/>
+      <c r="B12" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="C12" s="6"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C13" s="6"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C14" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2901,347 +2791,347 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="G1" s="5"/>
     </row>
     <row r="2" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>39</v>
+        <v>28</v>
+      </c>
+      <c r="F2" s="17" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>43</v>
+        <v>32</v>
+      </c>
+      <c r="F3" s="13" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>45</v>
-      </c>
       <c r="D4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="22" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="16" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="F5" s="26" t="s">
-        <v>50</v>
+      <c r="C5" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="23" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>52</v>
+        <v>28</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>55</v>
+        <v>28</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>57</v>
-      </c>
       <c r="D8" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" s="17" t="s">
-        <v>58</v>
+        <v>28</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>62</v>
+        <v>51</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>66</v>
+        <v>28</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>68</v>
+        <v>32</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>69</v>
-      </c>
       <c r="C12" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="F12" s="16" t="s">
-        <v>70</v>
+        <v>51</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>72</v>
+        <v>51</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>74</v>
+        <v>51</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -3269,854 +3159,831 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.88671875" style="28" customWidth="1"/>
-    <col min="2" max="2" width="45.5546875" style="7" customWidth="1"/>
+    <col min="1" max="1" width="19.88671875" style="24" customWidth="1"/>
+    <col min="2" max="2" width="45.5546875" style="6" customWidth="1"/>
     <col min="3" max="3" width="90.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="52.109375" style="7" customWidth="1"/>
-    <col min="5" max="5" width="28.6640625" style="29" customWidth="1"/>
-    <col min="6" max="6" width="28.6640625" style="7" customWidth="1"/>
-    <col min="7" max="7" width="48.6640625" style="29" customWidth="1"/>
-    <col min="8" max="8" width="25" style="7" customWidth="1"/>
-    <col min="9" max="9" width="47" style="7" customWidth="1"/>
-    <col min="10" max="10" width="77.6640625" style="7" customWidth="1"/>
-    <col min="11" max="11" width="58.88671875" style="7" customWidth="1"/>
-    <col min="12" max="16384" width="9.109375" style="29"/>
+    <col min="4" max="4" width="52.109375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="28.6640625" style="25" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="48.6640625" style="25" customWidth="1"/>
+    <col min="8" max="8" width="25" style="6" customWidth="1"/>
+    <col min="9" max="9" width="47" style="6" customWidth="1"/>
+    <col min="10" max="10" width="77.6640625" style="6" customWidth="1"/>
+    <col min="11" max="11" width="58.88671875" style="6" customWidth="1"/>
+    <col min="12" max="16384" width="9.109375" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="82.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:11" s="31" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
+    <row r="2" spans="1:11" s="27" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>78</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>79</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="E2" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="F2" s="26" t="s">
+        <v>82</v>
+      </c>
+      <c r="G2" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="H2" s="26" t="s">
+        <v>84</v>
+      </c>
+      <c r="I2" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="J2" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="K2" s="35" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="30" t="s">
-        <v>88</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="D2" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="E2" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="F2" s="30" t="s">
+    </row>
+    <row r="3" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="G2" s="30" t="s">
+      <c r="B3" s="28" t="s">
         <v>93</v>
       </c>
-      <c r="H2" s="30" t="s">
+      <c r="C3" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="I2" s="30" t="s">
+      <c r="D3" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="J2" s="39" t="s">
+      <c r="E3" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="K2" s="39" t="s">
+      <c r="F3" s="6" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="141.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="G3" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="H3" s="29" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="I3" s="30" t="s">
         <v>100</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="E3" s="6" t="s">
+    </row>
+    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="B4" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="28" t="s">
+      <c r="D4" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="E4" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="G4" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H4" s="29" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="I4" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="E4" s="29" t="s">
+      <c r="J4" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="F4" s="7" t="s">
+    </row>
+    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A5" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="B5" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="H4" s="33" t="s">
+      <c r="C5" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="I4" s="34" t="s">
+      <c r="D5" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="E5" s="25" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="28" t="s">
+      <c r="F5" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="H5" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="I5" s="29" t="s">
         <v>117</v>
       </c>
-      <c r="D5" s="7" t="s">
+    </row>
+    <row r="6" spans="1:11" ht="60.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="E5" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="F5" s="7" t="s">
+      <c r="B6" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="G5" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="H5" s="33" t="s">
+      <c r="D6" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="I5" s="33" t="s">
+      <c r="E6" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="H6" s="29" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A6" s="28" t="s">
+      <c r="I6" s="29" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="J6" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C6" s="5" t="s">
+    </row>
+    <row r="7" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A7" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="B7" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="E6" s="29" t="s">
+      <c r="C7" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="F6" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="G6" s="7" t="s">
+      <c r="D7" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="H6" s="33" t="s">
+      <c r="E7" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="H7" s="29" t="s">
         <v>129</v>
       </c>
-      <c r="I6" s="33" t="s">
+      <c r="I7" s="30" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="60.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="28" t="s">
+      <c r="J7" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B7" s="18" t="s">
-        <v>124</v>
-      </c>
-      <c r="C7" s="5" t="s">
+      <c r="K7" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="D7" s="7" t="s">
+    </row>
+    <row r="8" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="24" t="s">
         <v>133</v>
       </c>
-      <c r="E7" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="G7" s="7" t="s">
+      <c r="B8" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="H7" s="33" t="s">
+      <c r="C8" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="I7" s="33" t="s">
+      <c r="D8" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="E8" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="H8" s="29" t="s">
+        <v>129</v>
+      </c>
+      <c r="I8" s="30" t="s">
+        <v>130</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A9" s="24" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A8" s="28" t="s">
+      <c r="B9" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C9" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D9" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="E9" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G9" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="E8" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="H8" s="33" t="s">
+      <c r="H9" s="29" t="s">
+        <v>129</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>130</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="I8" s="34" t="s">
+      <c r="K9" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="J8" s="3" t="s">
+    </row>
+    <row r="10" spans="1:11" ht="59.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="24" t="s">
         <v>144</v>
       </c>
-      <c r="K8" s="7" t="s">
+      <c r="B10" s="15" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="28" t="s">
+      <c r="C10" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="D10" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E10" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="F10" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G10" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="H10" s="29" t="s">
         <v>149</v>
       </c>
-      <c r="E9" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="H9" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="I9" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="28" t="s">
+      <c r="I10" s="31" t="s">
         <v>150</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="J10" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C10" s="7" t="s">
+    </row>
+    <row r="11" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="24" t="s">
         <v>152</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="B11" s="15" t="s">
         <v>153</v>
       </c>
-      <c r="E10" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="G10" s="7" t="s">
+      <c r="C11" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="H10" s="33" t="s">
-        <v>142</v>
-      </c>
-      <c r="I10" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="J10" s="3" t="s">
+      <c r="D11" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="E11" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="F11" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G11" s="6" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" ht="59.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="28" t="s">
+      <c r="H11" s="32" t="s">
         <v>157</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="I11" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="J11" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="E11" s="29" t="s">
+    </row>
+    <row r="12" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A12" s="24" t="s">
         <v>160</v>
       </c>
-      <c r="F11" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G11" s="7" t="s">
+      <c r="B12" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="H11" s="33" t="s">
+      <c r="C12" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="I11" s="35" t="s">
+      <c r="D12" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="J11" s="3" t="s">
+      <c r="E12" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F12" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="H12" s="29" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A12" s="28" t="s">
+      <c r="I12" s="31" t="s">
         <v>165</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="J12" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="C12" s="5" t="s">
+    </row>
+    <row r="13" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="B13" s="15" t="s">
         <v>168</v>
       </c>
-      <c r="E12" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="F12" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G12" s="7" t="s">
+      <c r="C13" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="H12" s="36" t="s">
+      <c r="D13" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="I12" s="33" t="s">
+      <c r="E13" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F13" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="H13" s="29" t="s">
         <v>171</v>
       </c>
-      <c r="J12" s="13" t="s">
+      <c r="I13" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="J13" s="3" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="28" t="s">
+    <row r="14" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="24" t="s">
         <v>173</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B14" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D14" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="E13" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F13" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G13" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H13" s="33" t="s">
+      <c r="E14" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F14" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="H14" s="29" t="s">
         <v>177</v>
       </c>
-      <c r="I13" s="35" t="s">
+      <c r="I14" s="31" t="s">
+        <v>165</v>
+      </c>
+      <c r="J14" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="J13" s="3" t="s">
+    </row>
+    <row r="15" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="24" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
+      <c r="B15" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="C15" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="E15" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F15" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="H15" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="E14" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F14" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G14" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H14" s="33" t="s">
+      <c r="I15" s="29"/>
+      <c r="J15" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="I14" s="33" t="s">
-        <v>171</v>
-      </c>
-      <c r="J14" s="3" t="s">
+      <c r="K15" s="43" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="28" t="s">
+    <row r="16" spans="1:11" s="39" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16" s="24" t="s">
         <v>186</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B16" s="37" t="s">
         <v>187</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C16" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D16" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="E16" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="F16" s="40" t="s">
+        <v>106</v>
+      </c>
+      <c r="G16" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="H16" s="38" t="s">
         <v>189</v>
       </c>
-      <c r="E15" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F15" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H15" s="33" t="s">
+      <c r="I16" s="38" t="s">
         <v>190</v>
       </c>
-      <c r="I15" s="35" t="s">
-        <v>178</v>
-      </c>
-      <c r="J15" s="3" t="s">
+      <c r="J16" s="38" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="28" t="s">
+      <c r="K16" s="43"/>
+    </row>
+    <row r="17" spans="1:11" s="39" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="24" t="s">
         <v>192</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B17" s="37" t="s">
         <v>193</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C17" s="37" t="s">
         <v>194</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D17" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="E17" s="39" t="s">
+        <v>114</v>
+      </c>
+      <c r="F17" s="40" t="s">
+        <v>106</v>
+      </c>
+      <c r="G17" s="37" t="s">
         <v>195</v>
       </c>
-      <c r="E16" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F16" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H16" s="33" t="s">
+      <c r="H17" s="38" t="s">
         <v>196</v>
       </c>
-      <c r="I16" s="33"/>
-      <c r="J16" s="3" t="s">
+      <c r="I17" s="38" t="s">
         <v>197</v>
       </c>
-      <c r="K16" s="47" t="s">
+      <c r="J17" s="41" t="s">
         <v>198</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" s="43" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="28" t="s">
+      <c r="K17" s="43"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="24" t="s">
         <v>199</v>
       </c>
-      <c r="B17" s="41" t="s">
+      <c r="B18" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="C17" s="41" t="s">
+      <c r="F18" s="36"/>
+      <c r="H18" s="29" t="s">
         <v>201</v>
       </c>
-      <c r="D17" s="42" t="s">
-        <v>176</v>
-      </c>
-      <c r="E17" s="43" t="s">
-        <v>127</v>
-      </c>
-      <c r="F17" s="44" t="s">
-        <v>119</v>
-      </c>
-      <c r="G17" s="41" t="s">
-        <v>128</v>
-      </c>
-      <c r="H17" s="42" t="s">
+      <c r="I18" s="29" t="s">
         <v>202</v>
       </c>
-      <c r="I17" s="42" t="s">
+    </row>
+    <row r="19" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="24" t="s">
         <v>203</v>
       </c>
-      <c r="J17" s="42" t="s">
+      <c r="C19" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="K17" s="47"/>
-    </row>
-    <row r="18" spans="1:11" s="43" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A18" s="28" t="s">
+      <c r="D19" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="B18" s="41" t="s">
+      <c r="E19" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F19" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G19" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="C18" s="41" t="s">
+      <c r="H19" s="29" t="s">
+        <v>201</v>
+      </c>
+      <c r="I19" s="29" t="s">
         <v>207</v>
       </c>
-      <c r="D18" s="42" t="s">
-        <v>176</v>
-      </c>
-      <c r="E18" s="43" t="s">
-        <v>127</v>
-      </c>
-      <c r="F18" s="44" t="s">
-        <v>119</v>
-      </c>
-      <c r="G18" s="41" t="s">
+      <c r="J19" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="H18" s="42" t="s">
+    </row>
+    <row r="20" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A20" s="24" t="s">
         <v>209</v>
       </c>
-      <c r="I18" s="42" t="s">
+      <c r="B20" s="15" t="s">
         <v>210</v>
       </c>
-      <c r="J18" s="45" t="s">
+      <c r="C20" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="K18" s="47"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="28" t="s">
+      <c r="D20" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="E20" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F20" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="H20" s="29" t="s">
         <v>212</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="I20" s="32" t="s">
         <v>213</v>
       </c>
-      <c r="F19" s="40"/>
-      <c r="H19" s="33" t="s">
+      <c r="J20" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="I19" s="33" t="s">
+    </row>
+    <row r="21" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="24" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A20" s="28" t="s">
+      <c r="B21" s="15"/>
+      <c r="C21" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D21" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="E21" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="F21" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="H21" s="29" t="s">
         <v>218</v>
       </c>
-      <c r="E20" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F20" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G20" s="7" t="s">
+      <c r="I21" s="32"/>
+      <c r="K21" s="43" t="s">
         <v>219</v>
       </c>
-      <c r="H20" s="33" t="s">
-        <v>214</v>
-      </c>
-      <c r="I20" s="33" t="s">
+    </row>
+    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="24" t="s">
         <v>220</v>
       </c>
-      <c r="J20" s="7" t="s">
+      <c r="B22" s="15"/>
+      <c r="C22" s="5" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A21" s="28" t="s">
+      <c r="D22" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="E22" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="F22" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G22" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="H22" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="I22" s="32"/>
+      <c r="K22" s="43"/>
+    </row>
+    <row r="23" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="24" t="s">
         <v>224</v>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="E21" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F21" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="H21" s="33" t="s">
+      <c r="B23" s="15"/>
+      <c r="C23" s="34" t="s">
         <v>225</v>
       </c>
-      <c r="I21" s="36" t="s">
+      <c r="D23" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="J21" s="3" t="s">
+      <c r="E23" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="F23" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G23" s="6" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A22" s="28" t="s">
+      <c r="H23" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="I23" s="32"/>
+      <c r="K23" s="43"/>
+    </row>
+    <row r="24" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="24" t="s">
         <v>228</v>
       </c>
-      <c r="B22" s="18"/>
-      <c r="C22" s="5" t="s">
+      <c r="B24" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D24" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="E24" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F24" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G24" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="E22" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="F22" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G22" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="H22" s="33" t="s">
+      <c r="H24" s="29" t="s">
         <v>231</v>
       </c>
-      <c r="I22" s="36"/>
-      <c r="K22" s="47" t="s">
+      <c r="I24" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="J24" s="3" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="28" t="s">
+    <row r="25" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A25" s="24" t="s">
         <v>233</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="5" t="s">
+      <c r="B25" s="15" t="s">
         <v>234</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="C25" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="E23" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="F23" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G23" s="7" t="s">
+      <c r="D25" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="H23" s="33" t="s">
-        <v>231</v>
-      </c>
-      <c r="I23" s="36"/>
-      <c r="K23" s="47"/>
-    </row>
-    <row r="24" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="28" t="s">
+      <c r="E25" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F25" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="H25" s="32" t="s">
         <v>237</v>
       </c>
-      <c r="B24" s="18"/>
-      <c r="C24" s="38" t="s">
+      <c r="I25" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="J25" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="K25" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="E24" s="29" t="s">
-        <v>160</v>
-      </c>
-      <c r="F24" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G24" s="7" t="s">
+    </row>
+    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="24" t="s">
         <v>240</v>
       </c>
-      <c r="H24" s="33" t="s">
-        <v>231</v>
-      </c>
-      <c r="I24" s="36"/>
-      <c r="K24" s="47"/>
-    </row>
-    <row r="25" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A25" s="28" t="s">
+      <c r="B26" s="15" t="s">
         <v>241</v>
       </c>
-      <c r="B25" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="C25" s="5" t="s">
+      <c r="C26" s="5" t="s">
         <v>242</v>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="E25" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F25" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G25" s="7" t="s">
+      <c r="D26" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="H25" s="33" t="s">
+      <c r="E26" s="25" t="s">
+        <v>114</v>
+      </c>
+      <c r="F26" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="H26" s="32" t="s">
+        <v>237</v>
+      </c>
+      <c r="I26" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="J26" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="I25" s="33" t="s">
-        <v>130</v>
-      </c>
-      <c r="J25" s="3" t="s">
+      <c r="K26" s="6" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A26" s="28" t="s">
-        <v>246</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>247</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="D26" s="7" t="s">
-        <v>249</v>
-      </c>
-      <c r="E26" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F26" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="H26" s="36" t="s">
-        <v>250</v>
-      </c>
-      <c r="I26" s="33" t="s">
-        <v>171</v>
-      </c>
-      <c r="J26" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="K26" s="7" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="28" t="s">
-        <v>253</v>
-      </c>
-      <c r="B27" s="18" t="s">
-        <v>254</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="E27" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F27" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="H27" s="36" t="s">
-        <v>250</v>
-      </c>
-      <c r="I27" s="33" t="s">
-        <v>171</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="K27" s="7" t="s">
-        <v>258</v>
-      </c>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B27" s="15"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B28" s="18"/>
+      <c r="B28" s="15"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B29" s="18"/>
+      <c r="B29" s="15"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B30" s="18"/>
+      <c r="B30" s="15"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B31" s="18"/>
+      <c r="B31" s="15"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B32" s="18"/>
+      <c r="B32" s="15"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B33" s="18"/>
+      <c r="B33" s="15"/>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B34" s="18"/>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B35" s="18"/>
+      <c r="B34" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="K22:K24"/>
-    <mergeCell ref="K16:K18"/>
+    <mergeCell ref="K21:K23"/>
+    <mergeCell ref="K15:K17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4130,92 +3997,92 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="29"/>
-    <col min="2" max="2" width="40.5546875" style="29" customWidth="1"/>
-    <col min="3" max="3" width="83.44140625" style="29" customWidth="1"/>
-    <col min="4" max="4" width="32.44140625" style="7" customWidth="1"/>
-    <col min="5" max="16384" width="9.109375" style="29"/>
+    <col min="1" max="1" width="9.109375" style="25"/>
+    <col min="2" max="2" width="40.5546875" style="25" customWidth="1"/>
+    <col min="3" max="3" width="83.44140625" style="25" customWidth="1"/>
+    <col min="4" max="4" width="32.44140625" style="6" customWidth="1"/>
+    <col min="5" max="16384" width="9.109375" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>247</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>248</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="42">
+        <v>46247</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>250</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="42">
+        <v>46247</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>253</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="244.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="42">
+        <v>46247</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>256</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="42">
+        <v>46247</v>
+      </c>
+      <c r="B5" s="25" t="s">
         <v>259</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="C5" s="25" t="s">
         <v>260</v>
       </c>
-      <c r="C1" s="29" t="s">
+    </row>
+    <row r="6" spans="1:4" ht="225" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="42">
+        <v>46247</v>
+      </c>
+      <c r="B6" s="25" t="s">
         <v>261</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A2" s="46">
-        <v>46247</v>
-      </c>
-      <c r="B2" s="29" t="s">
+      <c r="D6" s="6" t="s">
         <v>263</v>
-      </c>
-      <c r="C2" s="12" t="s">
-        <v>264</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="46">
-        <v>46247</v>
-      </c>
-      <c r="B3" s="29" t="s">
-        <v>266</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="244.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="46">
-        <v>46247</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>269</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>270</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="46">
-        <v>46247</v>
-      </c>
-      <c r="B5" s="29" t="s">
-        <v>272</v>
-      </c>
-      <c r="C5" s="29" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="225" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="46">
-        <v>46247</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>274</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>275</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>276</v>
       </c>
     </row>
   </sheetData>
@@ -4238,48 +4105,48 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>262</v>
+        <v>249</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>277</v>
+        <v>264</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>278</v>
+        <v>265</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>279</v>
+        <v>266</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>280</v>
+        <v>267</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -4310,27 +4177,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="177.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="10" t="s">
-        <v>281</v>
-      </c>
-      <c r="B1" s="19" t="s">
-        <v>282</v>
+      <c r="A1" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
-        <v>283</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>284</v>
+      <c r="A2" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>271</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="171" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
-        <v>285</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>286</v>
+      <c r="A3" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -4338,7 +4205,7 @@
       <c r="C8" s="5"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="8"/>
+      <c r="F8" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4346,14 +4213,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4564,21 +4429,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4603,9 +4467,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
DeviceUse: config update of the main page name
</commit_message>
<xml_diff>
--- a/input/requirements/DeviceUse.xlsx
+++ b/input/requirements/DeviceUse.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MichalCiszewski\Documents\Github\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E873502A-EC35-43DA-9917-5EA8F879914C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B3CC70A-F4FD-4030-AD9D-CC2A8DC81138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" firstSheet="2" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -48,7 +48,7 @@
     <author>tc={34562484-290B-4F2D-9790-FE82BD1E616C}</author>
   </authors>
   <commentList>
-    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{34562484-290B-4F2D-9790-FE82BD1E616C}">
+    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{34562484-290B-4F2D-9790-FE82BD1E616C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -2269,8 +2269,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96E5C6F6-FD6C-477B-B67D-E91A0233B27C}" name="Tabel1" displayName="Tabel1" ref="A2:B12" totalsRowShown="0">
-  <autoFilter ref="A2:B12" xr:uid="{96E5C6F6-FD6C-477B-B67D-E91A0233B27C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{96E5C6F6-FD6C-477B-B67D-E91A0233B27C}" name="Tabel1" displayName="Tabel1" ref="A2:B11" totalsRowShown="0">
+  <autoFilter ref="A2:B11" xr:uid="{96E5C6F6-FD6C-477B-B67D-E91A0233B27C}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{37EF08FA-B565-414A-A476-BC12FA6A1A1B}" name="Veld"/>
     <tableColumn id="3" xr3:uid="{DDB6E257-D214-4298-B27F-676B3675AD2B}" name="Beschrijving" dataDxfId="8"/>
@@ -2611,10 +2611,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="B10" dT="2026-07-09T09:29:17.34" personId="{7313A655-1F36-4FD7-A150-7E7D12B2EDEE}" id="{34562484-290B-4F2D-9790-FE82BD1E616C}" done="1">
+  <threadedComment ref="B9" dT="2026-07-09T09:29:17.34" personId="{7313A655-1F36-4FD7-A150-7E7D12B2EDEE}" id="{34562484-290B-4F2D-9790-FE82BD1E616C}" done="1">
     <text>Of, is dit concept wel bedoelt voor aanlevering LIR? Het zou wel kunnen, maar dan hebben we het over een andere use case dan zorg-zorg. We hebben het dan over zorg-overheid. bestaat zon use case al?</text>
   </threadedComment>
-  <threadedComment ref="B10" dT="2026-07-20T09:49:23.46" personId="{1A9903B1-95BB-4B80-8FB6-9CB6AE3DAE32}" id="{46A8CD43-C164-44C4-9E7B-D71ECE1B481A}" parentId="{34562484-290B-4F2D-9790-FE82BD1E616C}">
+  <threadedComment ref="B9" dT="2026-07-20T09:49:23.46" personId="{1A9903B1-95BB-4B80-8FB6-9CB6AE3DAE32}" id="{46A8CD43-C164-44C4-9E7B-D71ECE1B481A}" parentId="{34562484-290B-4F2D-9790-FE82BD1E616C}">
     <text>Zowel de bouwblokken Device als DeviceUse zijn nodig voor LIR</text>
   </threadedComment>
 </ThreadedComments>
@@ -2656,7 +2656,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -2686,84 +2686,80 @@
       </c>
       <c r="C3" s="12"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-    </row>
-    <row r="5" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="334.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="334.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="C7" s="19"/>
+    </row>
+    <row r="8" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="19"/>
-    </row>
-    <row r="9" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="20"/>
+    </row>
+    <row r="9" spans="1:3" ht="231" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="20"/>
-    </row>
-    <row r="10" spans="1:3" ht="231" customHeight="1" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="C9" s="11"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="11" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="C10" s="11"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="11"/>
+        <v>274</v>
+      </c>
+      <c r="C11" s="6"/>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>274</v>
-      </c>
       <c r="C12" s="6"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C13" s="6"/>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C14" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4213,12 +4209,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4429,20 +4427,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -4467,12 +4466,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>